<commit_message>
docs: plan v3 probe-fix notes (s05/s07/s11); analysis: analyze_s14.py summary script
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
(cherry picked from commit 4622e7a5e7e53b66d3b61f9bd7f92a00fa114280)
</commit_message>
<xml_diff>
--- a/docs/proposals/NA_scenario_plan_2026-09-18_v3.xlsx
+++ b/docs/proposals/NA_scenario_plan_2026-09-18_v3.xlsx
@@ -1059,7 +1059,7 @@
       </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>5A -&gt; data scenario NorthAmerica_s05_brakes, run fel2026_s05_brakes_49_2015_v6. Regional DC multipliers on the post-2026 increment; GasPlants USA new-build cap 10 GW/yr 2027-31 (group cap); gas guardrail minimum = residual; RES rep funnel max without the x1.30 widening.</t>
+          <t>5A -&gt; data scenario NorthAmerica_s05_brakes, run fel2026_s05_brakes_49_2015_v6. Regional DC multipliers on the post-2026 increment; GasPlants USA new-build cap 10 GW/yr 2027-31 (group cap); gas guardrail minimum = residual; RES rep funnel max without the x1.30 widening (floored at the running maximum of the base minima - offshore pipelines and onshore floors would otherwise clash; found by the 1924 probe).</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>7C -&gt; data scenario NorthAmerica_s07_tech, run fel2026_s07_tech_49_2015_v6. SMR max 2/5/15/40 GW (2030/32/35/40), capex 5,090-&gt;3,330 EUR/kW; iron-air D_IronAir/S_IronAir (100 h, RTE 45 %, 60-&gt;20 USD/kWh, NA build cap 0.5-&gt;5 GW/yr); Li-ion optimistic rows reused; P_Fusion bull ramp min = max = 2.0/4.25/6.75/9.5 GW (2034/36/38/40).</t>
+          <t>7C -&gt; data scenario NorthAmerica_s07_tech, run fel2026_s07_tech_49_2015_v6. SMR max 2/5/15/40 GW (2030/32/35/40) but never below the base max/committed min (Darlington in Canada, probe fix), capex 5,090-&gt;3,330 EUR/kW; iron-air D_IronAir/S_IronAir (100 h, RTE 45 %, 60-&gt;20 USD/kWh, NA build cap 0.5-&gt;5 GW/yr); Li-ion optimistic rows reused; P_Fusion bull ramp min = max = 2.0/4.25/6.75/9.5 GW (2034/36/38/40).</t>
         </is>
       </c>
     </row>
@@ -1479,7 +1479,7 @@
       </c>
       <c r="N12" s="4" t="inlineStr">
         <is>
-          <t>11A -&gt; data scenario NorthAmerica_s11_feoc, run fel2026_s11_feoc_49_2015_v6. Li-ion capex x1.44 (2026) -&gt; x1.05 (2035); PV x1.02 2026-30; IC cost x1.2 whole horizon (no year dimension); LiIon USA cap 17 GW/yr 2026-27 (group cap).</t>
+          <t>11A -&gt; data scenario NorthAmerica_s11_feoc, run fel2026_s11_feoc_49_2015_v6. Li-ion capex x1.44 (2026) -&gt; x1.05 (2035); PV x1.02 2026-30; IC cost x1.2 whole horizon (no year dimension); LiIon USA cap 17 GW/yr 2026-27 (group cap); the base Li-ion forced-minimum path needs more than that in 2026-27, so the 2026/27 minima are scaled to the cap against the retiring residual fleet (16.7 / 33.3 GW cumulative new build), 2028+ minima unchanged (probe fix).</t>
         </is>
       </c>
     </row>

</xml_diff>